<commit_message>
Renames tab for webtool
</commit_message>
<xml_diff>
--- a/InputData/indst/IFStE/Indst Fuels Subject to Electrification.xlsx
+++ b/InputData/indst/IFStE/Indst Fuels Subject to Electrification.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us\InputData\indst\IFStE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB960117-6575-4783-A64A-41EB364DAC9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC8F182F-B3F9-4C66-BA27-F718955C1631}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-22845" yWindow="465" windowWidth="22590" windowHeight="14040" xr2:uid="{CEBBDD15-8244-44C2-A2EB-EB506D69E415}"/>
+    <workbookView xWindow="-4275" yWindow="-13455" windowWidth="17325" windowHeight="11040" xr2:uid="{CEBBDD15-8244-44C2-A2EB-EB506D69E415}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
-    <sheet name="IFStFS" sheetId="2" r:id="rId2"/>
+    <sheet name="IFStE" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -614,14 +614,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D74327C6-C2CB-4CD6-A944-44D7EC17E747}">
   <dimension ref="A1:C21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -629,69 +629,69 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>5</v>
       </c>
@@ -708,13 +708,13 @@
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:M26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="46.28515625" customWidth="1"/>
-    <col min="2" max="13" width="13.140625" customWidth="1"/>
+    <col min="1" max="1" width="46.26953125" customWidth="1"/>
+    <col min="2" max="13" width="13.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="5" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" s="5" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>7</v>
       </c>
@@ -755,7 +755,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -796,7 +796,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -837,7 +837,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -878,7 +878,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -919,7 +919,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -960,7 +960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -1001,7 +1001,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -1042,7 +1042,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -1083,7 +1083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -1124,7 +1124,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -1165,7 +1165,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>18</v>
       </c>
@@ -1206,7 +1206,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -1247,7 +1247,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>20</v>
       </c>
@@ -1288,7 +1288,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>21</v>
       </c>
@@ -1329,7 +1329,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -1370,7 +1370,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>23</v>
       </c>
@@ -1411,7 +1411,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>24</v>
       </c>
@@ -1452,7 +1452,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>25</v>
       </c>
@@ -1493,7 +1493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>26</v>
       </c>
@@ -1534,7 +1534,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>27</v>
       </c>
@@ -1575,7 +1575,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>28</v>
       </c>
@@ -1616,7 +1616,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>29</v>
       </c>
@@ -1657,7 +1657,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>30</v>
       </c>
@@ -1698,7 +1698,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>31</v>
       </c>
@@ -1739,7 +1739,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>32</v>
       </c>

</xml_diff>